<commit_message>
Usabilidade, melhorias no app e versão 2 do documento teórico (29-10-2026)
- Avaliação de usabilidade: 12 respostas com termo (média 4,79), análise em
  docs/evidencias_testes/usabilidade/
- App: entrada sem senha (nome opcional), legenda das cores no mapa, explicação
  do nível no cadastro e endereço aproximado nos detalhes
- Dados de demonstração com os centros dos bairros corrigidos
- Capturas refeitas (perfil "João Pedro"), PT-001 v1.5 (29/29 aprovados)
- Documento teórico versão 2 (67 páginas) e versão enviada ao orientador em 17/10
- CRONOGRAMA_STATUS.md, CLAUDE.md e seções T16 atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plano_e_fluxo_de_testes_TCC.xlsx
+++ b/docs/plano_e_fluxo_de_testes_TCC.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
     </row>
@@ -893,12 +893,12 @@
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>Em Andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>Sem sistema de autenticação de usuário implementado (fora do escopo do projeto); validar apenas navegação e leiaute com o público-alvo. Navegação verificada em 03/10/2026 (emulador, API real); falta a avaliação com o público-alvo.</t>
+          <t>Sem sistema de autenticação de usuário implementado (fora do escopo do projeto); validar apenas navegação e leiaute com o público-alvo. Navegação verificada em 03/10/2026 (emulador, API real); falta a avaliação com o público-alvo. 29/10/2026: avaliação de usabilidade concluída (12 participantes, média 4,79 em 5), ver docs/evidencias_testes/usabilidade/.</t>
         </is>
       </c>
     </row>
@@ -935,12 +935,12 @@
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>Em Andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>Cadastro integrado ao endpoint POST /ocorrencias real; ocorrência enviada é persistida no backend. Integração com POST /ocorrencias verificada em 03/10/2026 (CT-CAD-001/002/003); falta a avaliação com o público-alvo. 07/10/2026: busca por endereço, mapa arrastável e bloqueio de locais fora de São Caetano do Sul verificados (CT-CAD-005/006/007).</t>
+          <t>Cadastro integrado ao endpoint POST /ocorrencias real; ocorrência enviada é persistida no backend. Integração com POST /ocorrencias verificada em 03/10/2026 (CT-CAD-001/002/003); falta a avaliação com o público-alvo. 07/10/2026: busca por endereço, mapa arrastável e bloqueio de locais fora de São Caetano do Sul verificados (CT-CAD-005/006/007). 29/10/2026: avaliação de usabilidade concluída (12 participantes, média 4,79 em 5), ver docs/evidencias_testes/usabilidade/.</t>
         </is>
       </c>
     </row>
@@ -977,12 +977,12 @@
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Em Andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>Listagem consome GET /ocorrencias real (com filtros); validar navegação e leitura pelo público-alvo. GET /ocorrencias real verificado em 03/10/2026 (CT-LST-001/002, BUG-001 corrigido); falta a avaliação com o público-alvo.</t>
+          <t>Listagem consome GET /ocorrencias real (com filtros); validar navegação e leitura pelo público-alvo. GET /ocorrencias real verificado em 03/10/2026 (CT-LST-001/002, BUG-001 corrigido); falta a avaliação com o público-alvo. 29/10/2026: avaliação de usabilidade concluída (12 participantes, média 4,79 em 5), ver docs/evidencias_testes/usabilidade/.</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>Em Andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>Marcadores carregados a partir de ocorrências reais retornadas pela API; validar usabilidade da visualização geoespacial. Desbloqueado em 07/10/2026 com o cadastro do SHA-1 do APK de teste na chave do Google Maps: marcadores, painel da ocorrência, navegação para os detalhes e marcação do local no cadastro verificados (CT-MAP-001/002, CT-CAD-001); falta a avaliação com o público-alvo.</t>
+          <t>Marcadores carregados a partir de ocorrências reais retornadas pela API; validar usabilidade da visualização geoespacial. Desbloqueado em 07/10/2026 com o cadastro do SHA-1 do APK de teste na chave do Google Maps: marcadores, painel da ocorrência, navegação para os detalhes e marcação do local no cadastro verificados (CT-MAP-001/002, CT-CAD-001); falta a avaliação com o público-alvo. 29/10/2026: avaliação de usabilidade concluída (12 participantes, média 4,79 em 5), ver docs/evidencias_testes/usabilidade/.</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>Em Andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>Dados reais da ocorrência selecionada (via GET /ocorrencias/{id}); validar clareza das informações exibidas. GET /ocorrencias/{id} real verificado em 03/10/2026 (CT-DET-001); falta a avaliação com o público-alvo.</t>
+          <t>Dados reais da ocorrência selecionada (via GET /ocorrencias/{id}); validar clareza das informações exibidas. GET /ocorrencias/{id} real verificado em 03/10/2026 (CT-DET-001); falta a avaliação com o público-alvo. 29/10/2026: avaliação de usabilidade concluída (12 participantes, média 4,79 em 5), ver docs/evidencias_testes/usabilidade/.</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>Em Andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>Tela de configurações/perfil do usuário, com persistência real de preferências. Persistência local do perfil verificada em 03/10/2026 (CT-CFG-001); falta a avaliação com o público-alvo.</t>
+          <t>Tela de configurações/perfil do usuário, com persistência real de preferências. Persistência local do perfil verificada em 03/10/2026 (CT-CFG-001); falta a avaliação com o público-alvo. 29/10/2026: avaliação de usabilidade concluída (12 participantes, média 4,79 em 5), ver docs/evidencias_testes/usabilidade/.</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>Em Andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>Aba Previsão com o risco AHP atual, os dados do cálculo e os avisos oficiais do INMET (piso da classe). Conferida com GET /risco em 03/10 e 07/10/2026 (CT-PRV-001/002); ícones ⓘ com a origem dos dados em 07/10/2026 (CT-PRV-003); falta a avaliação com o público-alvo.</t>
+          <t>Aba Previsão com o risco AHP atual, os dados do cálculo e os avisos oficiais do INMET (piso da classe). Conferida com GET /risco em 03/10 e 07/10/2026 (CT-PRV-001/002); ícones ⓘ com a origem dos dados em 07/10/2026 (CT-PRV-003); falta a avaliação com o público-alvo. 29/10/2026: avaliação de usabilidade concluída (12 participantes, média 4,79 em 5), ver docs/evidencias_testes/usabilidade/.</t>
         </is>
       </c>
     </row>
@@ -1898,34 +1898,34 @@
       </c>
       <c r="K11" s="8" t="inlineStr">
         <is>
-          <t>Funcional OK contra a API real, agora com o local marcado por toque no mapa do cadastro: POST /ocorrencias 201, ocorrência gravada no PostGIS com o ponto tocado (POINT(-46.56265 -23.61966), nível Médio, id_usuario do perfil) e app abriu os detalhes. Avaliação de usabilidade com participantes externos ainda pendente.</t>
+          <t>Parte funcional aprovada em emulador (ver evidências anteriores). Avaliação de usabilidade por questionário sobre as capturas das telas (Google Forms, 12 participantes que aceitaram o termo, 17 a 21/10/2026): tela Cadastro com média 4,77 em 5 (critério ≥ 4). 9 de 12 entenderam a diferença entre Automático e escolher o nível (2 em parte, 1 não). Melhoria aplicada em 29/10/2026: Explicação dos dois modos sempre visível; texto que citava pluviômetros corrigido.</t>
         </is>
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>Em Execução</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr"/>
       <c r="N11" s="8" t="inlineStr"/>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>docs/evidencias_testes/2026-10-07/04_cadastro_local_no_mapa.png; docs/evidencias_testes/2026-10-07/05_cadastro_enviado_detalhes.png</t>
+          <t>docs/evidencias_testes/2026-10-07/04_cadastro_local_no_mapa.png; docs/evidencias_testes/2026-10-07/05_cadastro_enviado_detalhes.png; docs/evidencias_testes/usabilidade/analise_usabilidade_2026-10-29.md; docs/evidencias_testes/usabilidade/respostas_formulario_2026-10.csv</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>João (automação adb no emulador)</t>
+          <t>Grupo (formulário) e João (análise e melhorias)</t>
         </is>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="R11" s="8" t="inlineStr">
         <is>
-          <t>03/10/2026: local marcado por GPS (mapa sem autorização). 07/10/2026: refeito marcando o local no mapa, depois do cadastro do SHA-1. Registros de teste apagados do banco depois.</t>
+          <t>03/10/2026: local marcado por GPS (mapa sem autorização). 07/10/2026: refeito marcando o local no mapa, depois do cadastro do SHA-1. Registros de teste apagados do banco depois. Avaliação sem uso do app pelos participantes (só as telas) e amostra de conveniência (familiares e amigos): ver limitações em T16_secao_metodologia_testes.md.</t>
         </is>
       </c>
     </row>
@@ -2064,32 +2064,36 @@
       </c>
       <c r="K13" s="8" t="inlineStr">
         <is>
-          <t>Funcional OK: aba Alertas lista as 30 ocorrências de demonstração vindas da API, com fonte, nível, coordenadas e tempo relativo corretos. Avaliação de usabilidade com participantes externos ainda pendente.</t>
+          <t>Parte funcional aprovada em emulador (ver evidências anteriores). Avaliação de usabilidade por questionário sobre as capturas das telas (Google Forms, 12 participantes que aceitaram o termo, 17 a 21/10/2026): tela Alertas com média 4,62 em 5 (critério ≥ 4). 12 de 12 acharam os filtros fáceis de combinar.</t>
         </is>
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>Em Execução</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr"/>
       <c r="N13" s="8" t="inlineStr"/>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>docs/evidencias_testes/2026-10-03/03_alertas_api_real.png</t>
+          <t>docs/evidencias_testes/2026-10-03/03_alertas_api_real.png; docs/evidencias_testes/usabilidade/analise_usabilidade_2026-10-29.md; docs/evidencias_testes/usabilidade/respostas_formulario_2026-10.csv</t>
         </is>
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>João (automação adb no emulador)</t>
+          <t>Grupo (formulário) e João (análise e melhorias)</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
-        </is>
-      </c>
-      <c r="R13" s="8" t="inlineStr"/>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>Avaliação sem uso do app pelos participantes (só as telas) e amostra de conveniência (familiares e amigos): ver limitações em T16_secao_metodologia_testes.md.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="36" customHeight="1" s="6">
       <c r="A14" s="8" t="inlineStr">
@@ -2240,34 +2244,34 @@
       </c>
       <c r="K15" s="8" t="inlineStr">
         <is>
-          <t>Funcional OK: mapa do Google carregado (sem 'Authorization failure' no logcat) com as 30 ocorrências de demonstração da API como marcadores coloridos por nível (cartão 'Situação atual': 9 alto, 8 médio, 13 baixo) e enquadramento em São Caetano do Sul. Posição conferida: marcador da ocorrência nº 879 em -23.6124, -46.5754, igual a GET /ocorrencias/879. Avaliação de usabilidade com participantes externos ainda pendente.</t>
+          <t>Parte funcional aprovada em emulador (ver evidências anteriores). Avaliação de usabilidade por questionário sobre as capturas das telas (Google Forms, 12 participantes que aceitaram o termo, 17 a 21/10/2026): tela Mapa com média 4,73 em 5 (critério ≥ 4). 10 de 12 entenderam cores e marcadores esmaecidos (2 só as cores). Melhoria aplicada em 29/10/2026: Resumo do mapa passou a servir de legenda das cores e a explicar os esmaecidos.</t>
         </is>
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>Em Execução</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr"/>
       <c r="N15" s="8" t="inlineStr"/>
       <c r="O15" s="8" t="inlineStr">
         <is>
-          <t>docs/evidencias_testes/2026-10-07/01_mapa_marcadores.png</t>
+          <t>docs/evidencias_testes/2026-10-07/01_mapa_marcadores.png; docs/evidencias_testes/usabilidade/analise_usabilidade_2026-10-29.md; docs/evidencias_testes/usabilidade/respostas_formulario_2026-10.csv</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
-          <t>João (automação adb no emulador)</t>
+          <t>Grupo (formulário) e João (análise e melhorias)</t>
         </is>
       </c>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="R15" s="8" t="inlineStr">
         <is>
-          <t>03/10/2026: Bloqueado (chave do Google Maps restrita a outros certificados). Desbloqueado em 07/10/2026 com o cadastro do SHA-1 do certificado de depuração do notebook de testes nas restrições da chave. Execução com as 30 ocorrências; desde 07/10/2026 o mapa mostra só as das últimas 24 h (CT-MAP-003).</t>
+          <t>03/10/2026: Bloqueado (chave do Google Maps restrita a outros certificados). Desbloqueado em 07/10/2026 com o cadastro do SHA-1 do certificado de depuração do notebook de testes nas restrições da chave. Execução com as 30 ocorrências; desde 07/10/2026 o mapa mostra só as das últimas 24 h (CT-MAP-003). Avaliação sem uso do app pelos participantes (só as telas) e amostra de conveniência (familiares e amigos): ver limitações em T16_secao_metodologia_testes.md.</t>
         </is>
       </c>
     </row>
@@ -2325,34 +2329,34 @@
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>Funcional OK: toque no marcador abre o painel da ocorrência (descrição, coordenadas, nível, fonte e data/hora) e o botão 'Ver detalhes' abre a tela de detalhes da mesma ocorrência (nº 879, dados iguais aos de GET /ocorrencias/879). Avaliação de usabilidade com participantes externos ainda pendente.</t>
+          <t>Parte funcional aprovada em emulador (ver evidências anteriores). Avaliação de usabilidade por questionário sobre as capturas das telas (Google Forms, 12 participantes que aceitaram o termo, 17 a 21/10/2026): tela Mapa com média 4,73 em 5 (critério ≥ 4). Navegação mapa → detalhes avaliada pelas capturas das duas telas (sem tarefa no app).</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>Em Execução</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr"/>
       <c r="N16" s="8" t="inlineStr"/>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>docs/evidencias_testes/2026-10-07/02_mapa_marcador_selecionado.png; docs/evidencias_testes/2026-10-07/03_mapa_para_detalhes.png</t>
+          <t>docs/evidencias_testes/2026-10-07/02_mapa_marcador_selecionado.png; docs/evidencias_testes/2026-10-07/03_mapa_para_detalhes.png; docs/evidencias_testes/usabilidade/analise_usabilidade_2026-10-29.md; docs/evidencias_testes/usabilidade/respostas_formulario_2026-10.csv</t>
         </is>
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>João (automação adb no emulador)</t>
+          <t>Grupo (formulário) e João (análise e melhorias)</t>
         </is>
       </c>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="R16" s="8" t="inlineStr">
         <is>
-          <t>A navegação tem dois passos (marcador → painel → 'Ver detalhes'), não um: o painel permite conferir a ocorrência antes de sair do mapa. Desbloqueado em 07/10/2026 (ver CT-MAP-001).</t>
+          <t>A navegação tem dois passos (marcador → painel → 'Ver detalhes'), não um: o painel permite conferir a ocorrência antes de sair do mapa. Desbloqueado em 07/10/2026 (ver CT-MAP-001). Avaliação sem uso do app pelos participantes (só as telas) e amostra de conveniência (familiares e amigos): ver limitações em T16_secao_metodologia_testes.md.</t>
         </is>
       </c>
     </row>
@@ -2410,12 +2414,12 @@
       </c>
       <c r="K17" s="8" t="inlineStr">
         <is>
-          <t>Funcional OK: GET /ocorrencias/{id} 200; tela exibe nº, descrição, nível, fonte, data/hora e coordenadas. Avaliação de usabilidade com participantes externos ainda pendente.</t>
+          <t>Parte funcional aprovada em emulador (ver evidências anteriores). Avaliação de usabilidade por questionário sobre as capturas das telas (Google Forms, 12 participantes que aceitaram o termo, 17 a 21/10/2026): tela Detalhes com média 4,90 em 5 (critério ≥ 4). 9 de 12 acharam as informações suficientes (3 sentiram falta de endereço/bairro). Melhoria aplicada em 29/10/2026: Endereço aproximado (rua e bairro) incluído.</t>
         </is>
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>Em Execução</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -2430,22 +2434,22 @@
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>docs/evidencias_testes/2026-10-03/05_cadastro_manual_detalhes.png</t>
+          <t>docs/evidencias_testes/2026-10-03/05_cadastro_manual_detalhes.png; docs/evidencias_testes/usabilidade/analise_usabilidade_2026-10-29.md; docs/evidencias_testes/usabilidade/respostas_formulario_2026-10.csv</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
-          <t>João (automação adb no emulador)</t>
+          <t>Grupo (formulário) e João (análise e melhorias)</t>
         </is>
       </c>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="R17" s="8" t="inlineStr">
         <is>
-          <t>BUG-002: com o aparelho em português, as coordenadas saíam '-23,6148, -46,5435' (vírgula decimal confundida com a separadora). Corrigido em 03/10/2026 (sempre ponto decimal) e reverificado em pt-BR.</t>
+          <t>BUG-002: com o aparelho em português, as coordenadas saíam '-23,6148, -46,5435' (vírgula decimal confundida com a separadora). Corrigido em 03/10/2026 (sempre ponto decimal) e reverificado em pt-BR. Avaliação sem uso do app pelos participantes (só as telas) e amostra de conveniência (familiares e amigos): ver limitações em T16_secao_metodologia_testes.md.</t>
         </is>
       </c>
     </row>
@@ -2589,34 +2593,34 @@
       </c>
       <c r="K19" s="8" t="inlineStr">
         <is>
-          <t>Funcional OK: bairro salvo no perfil e mantido depois de fechar e reabrir o app (cartão em Ajustes: 'Olímpico • São Caetano do Sul'). Avaliação de usabilidade com participantes externos ainda pendente.</t>
+          <t>Parte funcional aprovada em emulador (ver evidências anteriores). Avaliação de usabilidade por questionário sobre as capturas das telas (Google Forms, 12 participantes que aceitaram o termo, 17 a 21/10/2026): tela Ajustes com média 4,83 em 5 (critério ≥ 4). 11 de 12 acharam as opções claras (1 em parte).</t>
         </is>
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>Em Execução</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr"/>
       <c r="N19" s="8" t="inlineStr"/>
       <c r="O19" s="8" t="inlineStr">
         <is>
-          <t>docs/evidencias_testes/2026-10-03/07_perfil_persistido.png</t>
+          <t>docs/evidencias_testes/2026-10-03/07_perfil_persistido.png; docs/evidencias_testes/usabilidade/analise_usabilidade_2026-10-29.md; docs/evidencias_testes/usabilidade/respostas_formulario_2026-10.csv</t>
         </is>
       </c>
       <c r="P19" s="8" t="inlineStr">
         <is>
-          <t>João (automação adb no emulador)</t>
+          <t>Grupo (formulário) e João (análise e melhorias)</t>
         </is>
       </c>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="R19" s="8" t="inlineStr">
         <is>
-          <t>Perfil e preferências ficam só no aparelho (SharedPreferences) — o backend não tem tabela de usuários.</t>
+          <t>Perfil e preferências ficam só no aparelho (SharedPreferences) — o backend não tem tabela de usuários. Avaliação sem uso do app pelos participantes (só as telas) e amostra de conveniência (familiares e amigos): ver limitações em T16_secao_metodologia_testes.md.</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2642,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Acessar a tela de login e avançar para a área principal</t>
+          <t>Acessar a tela de entrada (sem cadastro nem senha desde 29/10/2026) e avançar para a área principal</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -2675,34 +2679,34 @@
       </c>
       <c r="K20" s="8" t="inlineStr">
         <is>
-          <t>Funcional OK: nome e senha quaisquer levam à área principal; sessão mantida ao reabrir o app. Avaliação de usabilidade com participantes externos ainda pendente.</t>
+          <t>Parte funcional aprovada em emulador (ver evidências anteriores). Avaliação de usabilidade por questionário sobre as capturas das telas (Google Forms, 12 participantes que aceitaram o termo, 17 a 21/10/2026): tela Entrada com média 4,90 em 5 (critério ≥ 4). 10 de 12 acharam claro o aviso de senha (2 mais ou menos). Melhoria aplicada em 29/10/2026: Campo de senha retirado: entrada sem cadastro nem senha, nome opcional.</t>
         </is>
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>Em Execução</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr"/>
       <c r="N20" s="8" t="inlineStr"/>
       <c r="O20" s="8" t="inlineStr">
         <is>
-          <t>docs/evidencias_testes/2026-10-03/01_login.png</t>
+          <t>docs/evidencias_testes/2026-10-03/01_login.png; docs/evidencias_testes/usabilidade/analise_usabilidade_2026-10-29.md; docs/evidencias_testes/usabilidade/respostas_formulario_2026-10.csv</t>
         </is>
       </c>
       <c r="P20" s="8" t="inlineStr">
         <is>
-          <t>João (automação adb no emulador)</t>
+          <t>Grupo (formulário) e João (análise e melhorias)</t>
         </is>
       </c>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="R20" s="8" t="inlineStr">
         <is>
-          <t>Login não implementa autenticação real; não faz parte do escopo do sistema.</t>
+          <t>Login não implementa autenticação real; não faz parte do escopo do sistema. Avaliação sem uso do app pelos participantes (só as telas) e amostra de conveniência (familiares e amigos): ver limitações em T16_secao_metodologia_testes.md.</t>
         </is>
       </c>
     </row>
@@ -3617,34 +3621,34 @@
       </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>Funcional OK: os 5 cartões de fonte e o cartão 'Como o risco é calculado' abrem com o texto previsto; rótulos sem a fonte entre parênteses. Avaliação com participantes externos pendente.</t>
+          <t>Parte funcional aprovada em emulador (ver evidências anteriores). Avaliação de usabilidade por questionário sobre as capturas das telas (Google Forms, 12 participantes que aceitaram o termo, 17 a 21/10/2026): tela Previsão com média 4,77 em 5 (critério ≥ 4). 11 de 12 entenderam o risco Baixo com aviso do INMET (1 em dúvida).</t>
         </is>
       </c>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>Em Execução</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="M31" s="8" t="n"/>
       <c r="N31" s="8" t="n"/>
       <c r="O31" s="8" t="inlineStr">
         <is>
-          <t>docs/evidencias_testes/2026-10-07/07_previsao_info_fonte_ana.png; docs/evidencias_testes/2026-10-07/08_previsao_info_risco.png</t>
+          <t>docs/evidencias_testes/2026-10-07/07_previsao_info_fonte_ana.png; docs/evidencias_testes/2026-10-07/08_previsao_info_risco.png; docs/evidencias_testes/usabilidade/analise_usabilidade_2026-10-29.md; docs/evidencias_testes/usabilidade/respostas_formulario_2026-10.csv</t>
         </is>
       </c>
       <c r="P31" s="8" t="inlineStr">
         <is>
-          <t>João (automação adb no emulador)</t>
+          <t>Grupo (formulário) e João (análise e melhorias)</t>
         </is>
       </c>
       <c r="Q31" s="8" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
-          <t>Pedido do João em 07/10/2026: a origem dos dados e a explicação do cálculo saíram do texto da tela e foram para ícones ⓘ (área de toque de 48 dp, com descrição para leitor de tela).</t>
+          <t>Pedido do João em 07/10/2026: a origem dos dados e a explicação do cálculo saíram do texto da tela e foram para ícones ⓘ (área de toque de 48 dp, com descrição para leitor de tela). Avaliação sem uso do app pelos participantes (só as telas) e amostra de conveniência (familiares e amigos): ver limitações em T16_secao_metodologia_testes.md.</t>
         </is>
       </c>
     </row>

</xml_diff>